<commit_message>
Task 2: Integration Testing - controllers
</commit_message>
<xml_diff>
--- a/Exam/gymtrackerpro/lib/controller/__tests__/it/auth-controller/login-it-form.xlsx
+++ b/Exam/gymtrackerpro/lib/controller/__tests__/it/auth-controller/login-it-form.xlsx
@@ -14,9 +14,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="50">
-  <si>
-    <t>Statement: login(data: LoginUserInput): Promise&lt;ActionResult&lt;SessionData&gt;&gt; — validates input, delegates to AuthService, writes the returned session data into the session store, and returns an ActionResult.</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="52">
+  <si>
+    <t>Statement: login(data: LoginUserInput): Promise&lt;ActionResult&lt;SessionData&gt;&gt; - validates input, delegates to AuthService, writes the returned session data into the session store, and returns an ActionResult.</t>
   </si>
   <si>
     <t/>
@@ -34,13 +34,13 @@
     <t>Precondition</t>
   </si>
   <si>
-    <t>Database may or may not contain a user matching the supplied email. Session store is empty. All service and repository singletons are consumed from lib/di, which wires them against the shared PrismaClient instance. getSession() is mocked — it calls cookies() from next/headers which is a Next.js request-context primitive unavailable in Jest; the mock returns a controlled session object in its place.</t>
+    <t>Database may or may not contain a user matching the supplied email. Session store is empty.</t>
   </si>
   <si>
     <t>Results</t>
   </si>
   <si>
-    <t>ActionResult&lt;SessionData&gt; — { success: true, data: SessionData } on success. { success: false, message, errors? } on validation failure or any thrown error.</t>
+    <t>ActionResult&lt;SessionData&gt; - { success: true, data: SessionData } on success. { success: false, message, errors? } on validation failure or any thrown error.</t>
   </si>
   <si>
     <t>Postcondition</t>
@@ -58,6 +58,12 @@
     <t>Tear down:  npm run test:integration:down</t>
   </si>
   <si>
+    <t>All service and repository singletons are instantiated and accessed via the lib/di module, which configures them to use the shared PrismaClient instance.</t>
+  </si>
+  <si>
+    <t>getSession() is mocked as it calls cookies() from next/headers which is a Next.js request-context primitive unavailable in Jest; the mock returns a controlled session object in its place.</t>
+  </si>
+  <si>
     <t>No TC</t>
   </si>
   <si>
@@ -79,7 +85,7 @@
     <t>1</t>
   </si>
   <si>
-    <t xml:space="preserve">Member user seeded via userRepository.createMember (from lib/di).
+    <t xml:space="preserve">Member user seeded via userService.createMember (from lib/di).
 memberInput: { email: "member@gym.test", fullName: "Test Member", phone: "+40700000000", dateOfBirth: "1990-01-01", password: "ValidPass123!", membershipStart: "2024-01-01" }.
 mockSession satisfies Partial&lt;SessionData&gt; with save() and destroy() jest.fn().
 Input: { email: "member@gym.test", password: "ValidPass123!" }</t>
@@ -123,7 +129,7 @@
     <t>4</t>
   </si>
   <si>
-    <t xml:space="preserve">Member user seeded via userRepository.createMember (from lib/di) with password "ValidPass123!".
+    <t xml:space="preserve">Member user seeded via userService.createMember (from lib/di) with password "ValidPass123!".
 Input: { email: "member@gym.test", password: "WrongPass999!" }</t>
   </si>
   <si>
@@ -160,7 +166,7 @@
     <t>Re-tested</t>
   </si>
   <si>
-    <t>CTRL-1</t>
+    <t>CTRL-01</t>
   </si>
   <si>
     <t>n/a</t>
@@ -289,7 +295,7 @@
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="18364200" cy="4624387"/>
+    <xdr:ext cx="18873787" cy="5281612"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="1" name="Picture 1">
@@ -646,7 +652,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
@@ -681,7 +687,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" ht="95" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" ht="35" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>5</v>
       </c>
@@ -747,6 +753,22 @@
       </c>
       <c r="B13" s="1" t="s">
         <v>13</v>
+      </c>
+    </row>
+    <row r="14" ht="50" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="15" ht="50" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -763,7 +785,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A23"/>
+  <dimension ref="A1:A26"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="33" width="11" customWidth="1"/>
@@ -792,6 +814,9 @@
     <row r="21" ht="16" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="22" ht="16" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="23" ht="16" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="24" ht="16" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="25" ht="16" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="26" ht="16" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -817,22 +842,22 @@
         <v>1</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="2" ht="95" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -840,22 +865,22 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3" ht="35" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -863,22 +888,22 @@
         <v>1</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G3" s="6" t="s">
         <v>27</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="G3" s="6" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="4" ht="35" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -886,22 +911,22 @@
         <v>1</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C4" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F4" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="D4" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>29</v>
-      </c>
       <c r="G4" s="6" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" ht="50" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -909,22 +934,22 @@
         <v>1</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C5" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E5" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="D5" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>32</v>
-      </c>
       <c r="F5" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -952,17 +977,17 @@
         <v>1</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
       <c r="H4" s="2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="J4" s="2"/>
       <c r="K4" s="2"/>
@@ -974,40 +999,40 @@
         <v>1</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E5" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="J5" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="K5" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="L5" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="H5" s="4" t="s">
+      <c r="M5" s="4" t="s">
         <v>44</v>
-      </c>
-      <c r="I5" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="J5" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="K5" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="L5" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="M5" s="4" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
@@ -1015,7 +1040,7 @@
         <v>1</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C6" s="1">
         <v>4</v>
@@ -1027,28 +1052,28 @@
         <v>0</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="G6" s="1">
         <v>0</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="J6" s="1">
         <v>0</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="L6" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="M6" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>

</xml_diff>